<commit_message>
Add EEM fluorescence indices and Coble peak metrics
</commit_message>
<xml_diff>
--- a/examples/expected/示例数据_五区积分.xlsx
+++ b/examples/expected/示例数据_五区积分.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="积分结果" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行记录" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方法" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分区面积" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="荧光指标" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行记录" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="方法" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分区面积" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,32 +584,62 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>状态</t>
+          <t>BIX</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>说明</t>
+          <t>FI_470_520</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>一阶点数</t>
+          <t>HIX_Ohno</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>二阶点数</t>
+          <t>Peak_A_强度</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>插值点数</t>
+          <t>Peak_A_Em_nm</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>饱和点数</t>
+          <t>Peak_B_强度</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Peak_C_强度</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Peak_C_Em_nm</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Peak_M_强度</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Peak_M_Em_nm</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Peak_T_强度</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>备注</t>
         </is>
       </c>
     </row>
@@ -618,24 +649,40 @@
           <t>示例数据.xlsx</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>成功</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="B2" t="n">
+        <v>1.03830420230569</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.129481378350157</v>
+      </c>
       <c r="D2" t="n">
-        <v>333</v>
+        <v>0.3746773767526468</v>
       </c>
       <c r="E2" t="n">
-        <v>217</v>
+        <v>170.5</v>
       </c>
       <c r="F2" t="n">
-        <v>550</v>
+        <v>384</v>
       </c>
       <c r="G2" t="n">
-        <v>38</v>
-      </c>
+        <v>440.45</v>
+      </c>
+      <c r="H2" t="n">
+        <v>86.58</v>
+      </c>
+      <c r="I2" t="n">
+        <v>438</v>
+      </c>
+      <c r="J2" t="n">
+        <v>94.80799999999999</v>
+      </c>
+      <c r="K2" t="n">
+        <v>404</v>
+      </c>
+      <c r="L2" t="n">
+        <v>451.4</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -648,91 +695,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>项目</t>
+          <t>文件名</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>规则</t>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>一阶点数</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>二阶点数</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>插值点数</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>饱和点数</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>输入</t>
+          <t>示例数据.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sheet1 或首个工作表：首行 Ex、首列 Em；单调数值波长轴，可使用不同网格点数和间隔</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>插值</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>一阶 |Em−Ex|≤12 nm；二阶 |Em−(2Ex+4)|≤20 nm；沿 Ex 与 Em 双向线性插值取平均，插值负数截 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>积分</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>负数及 Em≤Ex 记 0；原仪器网格沿用二维梯形法，其他网格以三角网格线性插值并按边界裁剪积分</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>面积归一化</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PhiN_i=Phi_i×(本文件各区域总面积/本文件区域面积_i)；P_i=PhiN_i/sum(PhiN_i)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>分区边界</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>I: Ex≤250/Em≤330；II: Ex≤250/330–380；III: Ex≤250/Em≥380；IV: Ex≥250/Em≤380；V: Ex≥250/Em≥380</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>用途</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>插值点是估计值；不同扫描范围的 FRI 比例不可直接比较，应先统一波长范围</t>
-        </is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>333</v>
+      </c>
+      <c r="E2" t="n">
+        <v>217</v>
+      </c>
+      <c r="F2" t="n">
+        <v>550</v>
+      </c>
+      <c r="G2" t="n">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -746,6 +771,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>规则</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>输入</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>标准 XLSX/CSV：首行 Ex、首列 Em；可识别的岛津与 PicoQuant 原始 CSV；波长轴可使用不同点数和间隔</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>插值</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>一阶 |Em−Ex|≤12 nm；二阶 |Em−(2Ex+4)|≤20 nm；沿 Ex 与 Em 双向线性插值取平均，插值负数截 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>积分</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>负数及 Em≤Ex 记 0；原仪器网格沿用二维梯形法，其他网格以三角网格线性插值并按边界裁剪积分</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>面积归一化</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PhiN_i=Phi_i×(本文件各区域总面积/本文件区域面积_i)；P_i=PhiN_i/sum(PhiN_i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>分区边界</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>I: Ex≤250/Em≤330；II: Ex≤250/330–380；III: Ex≤250/Em≥380；IV: Ex≥250/Em≤380；V: Ex≥250/Em≥380</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>荧光指标数据</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>在瑞利散射插值后的矩阵计算；负强度记 0；非测量波长在原波长网格内线性插值，不外推</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BIX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>F(Ex310,Em380)/F(Ex310,Em430)；Huguet et al. 2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FI_470_520</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>F(Ex370,Em470)/F(Ex370,Em520)；使用 470/520 nm 版本，不是早期 450/500 nm 版本</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HIX_Ohno</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ex254 nm；H=Em435–480 nm 积分，L=Em300–345 nm 积分；HIX=H/(L+H)；Ohno 2002 归一化版本</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Peak_B、Peak_T</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B=F(Ex275,Em310)，T=F(Ex275,Em340)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Peak_A、Peak_M、Peak_C</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>固定 Ex 下按 Em 区间取峰值及峰位：A=Ex260/Em380–460；M=Ex312/Em380–420；C=Ex350/Em420–480 nm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>指标缺值</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>所需波长不在扫描范围，或比值分母为 0 时对应单元格留空；具体项见荧光指标的备注列</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>插值点是估计值；不同扫描范围的 FRI 比例不可直接比较，应先统一波长范围</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>